<commit_message>
data(fase10): refresh Genetic rows in BENCHMARK_CSV with tuned 60/80 GA
Only Genetic changed (every other strategy is deterministic/unchanged), so just
its existing rows were re-run, not the expensive KGeoMIP/KQNodes on n=15/20/25.
Big gains: N15A k=3 0.556 -> 0.054, N10A k=3 2.38 -> 0.96, N10A k=4 3.88 -> 2.39.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/results/benchmark_results_FINAL.xlsx
+++ b/data/results/benchmark_results_FINAL.xlsx
@@ -573,7 +573,7 @@
         <v>0.469727</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2406</v>
+        <v>0.5313</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -790,16 +790,16 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>2.380859</v>
+        <v>0.958008</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2437</v>
+        <v>0.9187</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>B1: f | ADH
-B2: abcdeghij | BCEFGJ
-B3: ∅ | I</t>
+          <t>B1: abcdefghij | ACEFGHIJ
+B2: ∅ | B
+B3: ∅ | D</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1017,16 +1017,16 @@
         <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>3.884766</v>
+        <v>2.391602</v>
       </c>
       <c r="F19" t="n">
-        <v>0.2498</v>
+        <v>0.7173</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>B1: i | A
-B2: abcegj | BCFJ
-B3: dfh | DEGH
+          <t>B1: f | AH
+B2: abcdeghij | BCEFGJ
+B3: ∅ | D
 B4: ∅ | I</t>
         </is>
       </c>
@@ -1242,15 +1242,15 @@
         <v>2</v>
       </c>
       <c r="E26" t="n">
-        <v>0.02679</v>
+        <v>0.027029</v>
       </c>
       <c r="F26" t="n">
-        <v>1.3231</v>
+        <v>4.2492</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>B1: abcdefghijklmno | ABCDEFGIJKLMNO
-B2: ∅ | H</t>
+          <t>B1: ∅ | A
+B2: abcdefghijklmno | BCDEFGHIJKLMNO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -1462,16 +1462,16 @@
         <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>0.556135</v>
+        <v>0.053899</v>
       </c>
       <c r="F33" t="n">
-        <v>1.6574</v>
+        <v>4.5085</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>B1: h | ∅
-B2: abcdefgijklmno | ABCDEFGHJKLMNO
-B3: ∅ | I</t>
+          <t>B1: abcdefghijklmno | ABCDEFGIKLMNO
+B2: ∅ | H
+B3: ∅ | J</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1689,17 +1689,17 @@
         <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>0.919816</v>
+        <v>0.833143</v>
       </c>
       <c r="F40" t="n">
-        <v>2.4428</v>
+        <v>6.5568</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>B1: cdefgijklmn | ABCHJLMN
-B2: b | DEIO
-B3: ∅ | F
-B4: aho | GK</t>
+          <t>B1: abcdefhijlno | ABCFHJLMN
+B2: m | DEK
+B3: k | G
+B4: g | IO</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -2310,10 +2310,10 @@
         <v>0.469727</v>
       </c>
       <c r="E8" t="n">
-        <v>2.380859</v>
+        <v>0.958008</v>
       </c>
       <c r="F8" t="n">
-        <v>3.884766</v>
+        <v>2.391602</v>
       </c>
     </row>
     <row r="9">
@@ -2326,13 +2326,13 @@
         <v>15</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02679</v>
+        <v>0.027029</v>
       </c>
       <c r="E9" t="n">
-        <v>0.556135</v>
+        <v>0.053899</v>
       </c>
       <c r="F9" t="n">
-        <v>0.919816</v>
+        <v>0.833143</v>
       </c>
     </row>
     <row r="10">

</xml_diff>